<commit_message>
Design verandering. Pcb -> niet
</commit_message>
<xml_diff>
--- a/documenten/beheer/Bestellijst-GSTEM.xlsx
+++ b/documenten/beheer/Bestellijst-GSTEM.xlsx
@@ -9,11 +9,11 @@
   <sheets>
     <sheet name="Bestellijst" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Legende" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Bestelschema PCB" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Bedrading en montage" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Bestelbaarheid" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$2:$J$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Bestellijst'!$A$2:$J$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -101,17 +101,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E1D5E7"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -121,7 +121,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E1D5E7"/>
       </patternFill>
     </fill>
     <fill>
@@ -170,7 +170,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -221,9 +221,6 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -237,11 +234,11 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -249,12 +246,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -639,7 +630,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Bestellijst G-Stem meettoestel - prijzen incl. btw (Kiwi + antratek + TME + Mouser + HESTORE + TinyTronics + AliExpress + AISLER, definitief 2026-10-07)</t>
+          <t>Bestellijst G-Stem meettoestel - prijzen incl. btw (Kiwi + antratek + TME + Mouser + AliExpress; bijgewerkt 2026-10-09)</t>
         </is>
       </c>
     </row>
@@ -1141,76 +1132,44 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Voeding</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>Voedingsaansluiting (op de print)</t>
-        </is>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>2,1 mm DC-barreljack, breadboard-/PCB-compatibel</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F16" s="8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="I16" s="10" t="inlineStr">
-        <is>
-          <t>https://www.kiwi-electronics.com/nl/2-1mm-dc-barrel-jack-breadboard-compatible-415</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>Naast de bestaande adapter; voor nette montage op de draagprint</t>
-        </is>
-      </c>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Vervallen ontwerp</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n"/>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
+      <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Voeding</t>
+          <t>Vervallen ontwerp</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Buck-converter 5 V</t>
+          <t>PCB-voedingsaansluiting</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Heeft de gebruiker</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>1</v>
-      </c>
+          <t>2,1 mm breadboard-/PCB-barreljack - alleen bedoeld voor de vervallen draagprint</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
-      <c r="G17" s="14" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
@@ -1221,55 +1180,25 @@
       <c r="I17" s="6" t="inlineStr"/>
       <c r="J17" s="6" t="inlineStr">
         <is>
-          <t>Referentie antratek: Buck Regulator Breakout 5V (EUR 12,04)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+          <t>Niet bestellen. De bestaande barrel-adapter blijft; voedingsinvoer via de behuizing nog te bepalen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Voeding</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>Bescherming voeding</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>2 A PTC Littelfuse 1812L200/16 + TVS SMBJ10A-TR (zonder P-MOSFET)</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="15" t="inlineStr">
-        <is>
-          <t>mouser</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>Mouser.be / DigiKey (EU-magazijn)</t>
-        </is>
-      </c>
-      <c r="I18" s="10" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Littelfuse/1812L200-16DR</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>PTC bij Mouser/DigiKey (EU); TVS SMBJ10A bij TME. P-MOSFET vervalt (beslissing 2026-10-06).</t>
-        </is>
-      </c>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+      <c r="E18" s="4" t="n"/>
+      <c r="F18" s="4" t="n"/>
+      <c r="G18" s="4" t="n"/>
+      <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1279,12 +1208,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Ompoolbeveiliging (P-MOSFET)</t>
+          <t>Buck-converter 5 V</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>P-MOSFET DMG2301L / AO3401A (SOT-23)</t>
+          <t>Heeft de gebruiker</t>
         </is>
       </c>
       <c r="D19" s="7" t="n">
@@ -1292,9 +1221,9 @@
       </c>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
-      <c r="G19" s="16" t="inlineStr">
-        <is>
-          <t>niet nodig</t>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1305,7 +1234,7 @@
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>BESLISSING 2026-10-06: NIET voorzien. Geen P-MOSFET-ompoolbeveiliging; voorkom omgekeerd aansluiten met een gepolariseerde connector (XT60/JST-XH). Zie data/afgevoerd.md.</t>
+          <t>Referentie antratek: Buck Regulator Breakout 5V (EUR 12,04)</t>
         </is>
       </c>
     </row>
@@ -1317,41 +1246,41 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>LDO 3,3 V</t>
+          <t>Bescherming voeding</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>AP2112K-3.3TRG1 (Diodes Inc., SOT-23-5)</t>
+          <t>2 A PTC Littelfuse 1812L200/16 + TVS SMBJ10A-TR (zonder P-MOSFET)</t>
         </is>
       </c>
       <c r="D20" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>0.27</v>
+        <v>1</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>tme</t>
+        <v>1</v>
+      </c>
+      <c r="G20" s="16" t="inlineStr">
+        <is>
+          <t>mouser</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>TME (Polen, EU)</t>
+          <t>Mouser.be / DigiKey (EU-magazijn)</t>
         </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
-          <t>https://www.tme.eu/en/details/ap2112k-3.3trg1/ldo-fixed-voltage-regulators/diodes-incorporated/</t>
+          <t>https://www.mouser.com/ProductDetail/Littelfuse/1812L200-16DR</t>
         </is>
       </c>
       <c r="J20" s="6" t="inlineStr">
         <is>
-          <t>8000+ op voorraad bij TME</t>
+          <t>PTC bij Mouser/DigiKey (EU); TVS SMBJ10A bij TME. P-MOSFET vervalt (beslissing 2026-10-06).</t>
         </is>
       </c>
     </row>
@@ -1363,18 +1292,20 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Aan/uit-schakelaar</t>
+          <t>Ompoolbeveiliging (P-MOSFET)</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Geen; toestel start bij voeding</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="n"/>
+          <t>P-MOSFET DMG2301L / AO3401A (SOT-23)</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
-      <c r="G21" s="16" t="inlineStr">
+      <c r="G21" s="15" t="inlineStr">
         <is>
           <t>niet nodig</t>
         </is>
@@ -1385,74 +1316,94 @@
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Draagprint (PCB bij AISLER)</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-      <c r="H22" s="4" t="n"/>
-      <c r="I22" s="4" t="n"/>
-      <c r="J22" s="4" t="n"/>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>BESLISSING 2026-10-06: NIET voorzien. Geen P-MOSFET-ompoolbeveiliging; voorkom omgekeerd aansluiten met een gepolariseerde connector (XT60/JST-XH). Zie data/afgevoerd.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Voeding</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>LDO 3,3 V</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>AP2112K-3.3TRG1 (Diodes Inc., SOT-23-5)</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>tme</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>TME (Polen, EU)</t>
+        </is>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>https://www.tme.eu/en/details/ap2112k-3.3trg1/ldo-fixed-voltage-regulators/diodes-incorporated/</t>
+        </is>
+      </c>
+      <c r="J22" s="6" t="inlineStr">
+        <is>
+          <t>8000+ op voorraad bij TME</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Draagprint (PCB bij AISLER)</t>
+          <t>Voeding</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Draagprint (printplaat)</t>
+          <t>Aan/uit-schakelaar</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>2-laags 1,6 mm HASL, set van 3 stuks - AISLER</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="E23" s="8" t="n">
-        <v>10.92</v>
-      </c>
-      <c r="F23" s="8" t="n">
-        <v>32.76</v>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>aisler</t>
+          <t>Geen; toestel start bij voeding</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>AISLER</t>
-        </is>
-      </c>
-      <c r="I23" s="10" t="inlineStr">
-        <is>
-          <t>https://aisler.net</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>Schatting 75 cm2 (100x75 mm), incl. btw; Budget-service. Formule: EUR 12,00 + EUR 0,067/cm2 x oppervlak x aantal. AISLER levert in sets van 3; gratis verzending. Definitieve maat volgt uit de KiCad-layout</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="6" t="inlineStr"/>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Print en verbindingen</t>
+          <t>Vervallen ontwerp</t>
         </is>
       </c>
       <c r="B24" s="4" t="n"/>
@@ -1468,165 +1419,123 @@
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Print en verbindingen</t>
+          <t>Vervallen ontwerp</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Level shifter 3,3 V &lt;-&gt; 5 V</t>
+          <t>Draagprint (carrier-PCB)</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>8-kanaals bidirectionele Logic Level Converter - TXB0108</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="8" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="F25" s="8" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="G25" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
+          <t>Eigen PCB bij AISLER</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="I25" s="10" t="inlineStr">
-        <is>
-          <t>https://www.kiwi-electronics.com/nl/8-channel-bi-directional-logic-level-converter-txb0108-836</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr"/>
       <c r="J25" s="6" t="inlineStr">
         <is>
-          <t>DEFINITIEF (2026-10-07): TXB0108-breakout. De TXB0104-IC (TSSOP-14, ca. EUR 1,80) is enkel een alternatief; antratek BSS138-converter EUR 4,78 is een ander type</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Print en verbindingen</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Schroefklem 4-pins 3,5 mm</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>DEGSON DG250-3.5-04P-11-00A(H) (push-in) of KF128 (schroef)</t>
-        </is>
-      </c>
-      <c r="D26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="8" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="F26" s="8" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="G26" s="18" t="inlineStr">
-        <is>
-          <t>hestore</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>HESTORE (HU, EU) / TME</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>https://www.hestore.eu/en/prod_10044104.html</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr">
-        <is>
-          <t>Kiwi heeft alleen 3-weg; de schroefvariant KF128 is in de EU minder courant</t>
-        </is>
-      </c>
+          <t>Vervallen op 2026-10-09: de gebruiker bedradt en soldeert de onderdelen zelf en monteert ze aan een 3D-geprinte behuizing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Bedrading en losse elektronica</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="n"/>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4" t="n"/>
+      <c r="G26" s="4" t="n"/>
+      <c r="H26" s="4" t="n"/>
+      <c r="I26" s="4" t="n"/>
+      <c r="J26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Print en verbindingen</t>
+          <t>Bedrading en losse elektronica</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Sockets</t>
+          <t>Level shifter 3,3 V &lt;-&gt; 5 V</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Dual-wipe female headers (XIAO + sensoren) + turned-pin precisie-sockets (vaste modules)</t>
+          <t>8-kanaals bidirectionele Logic Level Converter - TXB0108</t>
         </is>
       </c>
       <c r="D27" s="7" t="n">
         <v>1</v>
       </c>
       <c r="E27" s="8" t="n">
-        <v>5</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="G27" s="12" t="inlineStr">
-        <is>
-          <t>tme</t>
+        <v>8.699999999999999</v>
+      </c>
+      <c r="G27" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Mouser / DigiKey / TME</t>
+          <t>Kiwi Electronics</t>
         </is>
       </c>
       <c r="I27" s="10" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/connectors/headers-wire-housings/</t>
+          <t>https://www.kiwi-electronics.com/nl/8-channel-bi-directional-logic-level-converter-txb0108-836</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>Standaard 2,54 mm turned-pin/dual-wipe; Preci-Dip bij TME is business/MOQ 380 en valt af</t>
+          <t>DEFINITIEF (2026-10-07): TXB0108-breakout. De TXB0104-IC (TSSOP-14, ca. EUR 1,80) is enkel een alternatief; antratek BSS138-converter EUR 4,78 is een ander type</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Print en verbindingen</t>
+          <t>Bedrading en losse elektronica</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Power-LED + serieweerstand</t>
+          <t>UART-/uitbreidingsconnector</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>3 mm LED rood (10-pack) + weerstand 330 Ohm (10-pack) - heeft de gebruiker thuis</t>
-        </is>
-      </c>
-      <c r="D28" s="7" t="n">
-        <v>1</v>
-      </c>
+          <t>Eerder gekozen DEGSON 4-pins 3,5 mm; mogelijk overbodig bij rechtstreeks bedraden</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n"/>
       <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n"/>
-      <c r="G28" s="14" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>te bepalen</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
@@ -1637,256 +1546,226 @@
       <c r="I28" s="6" t="inlineStr"/>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>HEEFT DE GEBRUIKER THUIS (2026-10-06): 10-pack rode 3 mm LED + 10-pack 330 Ohm; niet aankopen. Referentie Kiwi: LED EUR 1,20 + weerstand EUR 0,96 = EUR 2,16</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Print en verbindingen</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>Ontkoppelcondensatoren</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Keramische condensator kit (15 soorten, 450 st.) - dekt 100 nF + 10 uF</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="8" t="n">
-        <v>10.27</v>
-      </c>
-      <c r="F29" s="8" t="n">
-        <v>10.27</v>
-      </c>
-      <c r="G29" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
-        </is>
-      </c>
-      <c r="H29" s="5" t="inlineStr">
-        <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="I29" s="10" t="inlineStr">
-        <is>
-          <t>https://www.kiwi-electronics.com/nl/keramische-condensator-kit-in-doos-15-soorten-450-stuks-10492</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="inlineStr">
-        <is>
-          <t>Kit i.p.v. losse condensatoren</t>
-        </is>
-      </c>
+          <t>Nog geen keuze of aankoop; eerst bevestigen hoe de kabel naar buiten wordt aangesloten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Vervallen ontwerp</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n"/>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="n"/>
+      <c r="F29" s="4" t="n"/>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="n"/>
+      <c r="J29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Print en verbindingen</t>
+          <t>Vervallen ontwerp</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Bulk-elco</t>
+          <t>Socket-headers</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>100 uF / 16 V op de 5 V-ingang</t>
-        </is>
-      </c>
-      <c r="D30" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="8" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="F30" s="8" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>kiwi</t>
+          <t>Dual-wipe en turned-pin sockets</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="I30" s="10" t="inlineStr">
-        <is>
-          <t>https://www.kiwi-electronics.com/nl/100uf-16v-condensator-440</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Print en verbindingen</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="inlineStr">
-        <is>
-          <t>I2C-pull-ups op de print</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>Niet nodig; breakouts hebben ze al</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="16" t="inlineStr">
-        <is>
-          <t>niet nodig</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr"/>
-      <c r="J31" s="6" t="inlineStr">
-        <is>
-          <t>2 reserve-footprints</t>
-        </is>
-      </c>
+      <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>Vervallen op 2026-10-09: breakoutmodules worden handbedraad en gesoldeerd; niet bestellen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Bedrading en losse elektronica</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n"/>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="n"/>
+      <c r="F31" s="4" t="n"/>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="n"/>
+      <c r="J31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Print en verbindingen</t>
+          <t>Bedrading en losse elektronica</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>Montage</t>
+          <t>Power-LED + serieweerstand</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>M3-schroeven, moeren, afstandsbusjes, nylon spacers</t>
+          <t>3 mm LED rood (10-pack) + weerstand 330 Ohm (10-pack) - heeft de gebruiker thuis</t>
         </is>
       </c>
       <c r="D32" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="F32" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="G32" s="11" t="inlineStr">
-        <is>
-          <t>tinytronics</t>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>TinyTronics (NL, EU)</t>
-        </is>
-      </c>
-      <c r="I32" s="10" t="inlineStr">
-        <is>
-          <t>https://www.tinytronics.nl/nl/gereedschap-en-montage/installatie-en-montagemateriaal/afstandsbusjes/m3-afstandsbusje-kit</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr"/>
       <c r="J32" s="6" t="inlineStr">
         <is>
-          <t>Alternatief: Bits &amp; Parts (NL) 180-delige M3-set EUR 6,95</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Kabels en verbruik (in bezit)</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
-      <c r="I33" s="4" t="n"/>
-      <c r="J33" s="4" t="n"/>
+          <t>HEEFT DE GEBRUIKER THUIS (2026-10-06): 10-pack rode 3 mm LED + 10-pack 330 Ohm; niet aankopen. Referentie Kiwi: LED EUR 1,20 + weerstand EUR 0,96 = EUR 2,16</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Bedrading en losse elektronica</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Ontkoppelcondensatoren</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Keramische condensator kit (15 soorten, 450 st.) - dekt 100 nF + 10 uF</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="8" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>10.27</v>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I33" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/keramische-condensator-kit-in-doos-15-soorten-450-stuks-10492</t>
+        </is>
+      </c>
+      <c r="J33" s="6" t="inlineStr">
+        <is>
+          <t>Kit i.p.v. losse condensatoren</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Kabels en verbruik (in bezit)</t>
+          <t>Bedrading en losse elektronica</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>USB-C datakabel</t>
+          <t>Bulk-elco</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Eigen kabel</t>
+          <t>100 uF / 16 V op de 5 V-ingang</t>
         </is>
       </c>
       <c r="D34" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="14" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
+      <c r="E34" s="8" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>kiwi</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I34" s="6" t="inlineStr"/>
+          <t>Kiwi Electronics</t>
+        </is>
+      </c>
+      <c r="I34" s="10" t="inlineStr">
+        <is>
+          <t>https://www.kiwi-electronics.com/nl/100uf-16v-condensator-440</t>
+        </is>
+      </c>
       <c r="J34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Kabels en verbruik (in bezit)</t>
+          <t>Bedrading en losse elektronica</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Dupont-/siliconendraad</t>
+          <t>I2C-pull-ups</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Heeft de gebruiker</t>
-        </is>
-      </c>
-      <c r="D35" s="7" t="n">
-        <v>1</v>
-      </c>
+          <t>Niet nodig; breakouts hebben ze al</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n"/>
       <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="n"/>
-      <c r="G35" s="14" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
+      <c r="G35" s="15" t="inlineStr">
+        <is>
+          <t>niet nodig</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -1895,106 +1774,112 @@
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
-      <c r="J35" s="6" t="inlineStr"/>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>Geen extra pull-ups voorzien.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Kabels en verbruik (in bezit)</t>
+          <t>Bedrading en losse elektronica</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>USB A-kabel LoRa-ontvanger</t>
+          <t>Behuizingsmontage</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>USB-A naar USB-C voor de XIAO (heeft de gebruiker)</t>
-        </is>
-      </c>
-      <c r="D36" s="7" t="n">
-        <v>1</v>
-      </c>
+          <t>Bevestigingsmateriaal nog te bepalen; eerdere M3-set was voor de draagprint</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n"/>
       <c r="E36" s="5" t="n"/>
       <c r="F36" s="5" t="n"/>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="G36" s="17" t="inlineStr">
+        <is>
+          <t>te bepalen</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr"/>
+      <c r="J36" s="6" t="inlineStr">
+        <is>
+          <t>Niet bestellen of online opzoeken voordat de gebruiker de montagewijze heeft bevestigd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Kabels en verbruik (in bezit)</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="n"/>
+      <c r="D37" s="4" t="n"/>
+      <c r="E37" s="4" t="n"/>
+      <c r="F37" s="4" t="n"/>
+      <c r="G37" s="4" t="n"/>
+      <c r="H37" s="4" t="n"/>
+      <c r="I37" s="4" t="n"/>
+      <c r="J37" s="4" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Kabels en verbruik (in bezit)</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>USB-C datakabel</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Eigen kabel</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="14" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
       </c>
-      <c r="H36" s="5" t="inlineStr">
+      <c r="H38" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I36" s="6" t="inlineStr"/>
-      <c r="J36" s="6" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>Kabels en verbruik (in bezit)</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>Gereedschap</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>Schuifmaat, soldeerbout, tin, flux, multimeter, USB-serieel adapter</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="14" t="inlineStr">
-        <is>
-          <t>al in bezit</t>
-        </is>
-      </c>
-      <c r="H37" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I37" s="6" t="inlineStr"/>
-      <c r="J37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Mock-up (vliegtuigje)</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="n"/>
-      <c r="C38" s="4" t="n"/>
-      <c r="D38" s="4" t="n"/>
-      <c r="E38" s="4" t="n"/>
-      <c r="F38" s="4" t="n"/>
-      <c r="G38" s="4" t="n"/>
-      <c r="H38" s="4" t="n"/>
-      <c r="I38" s="4" t="n"/>
-      <c r="J38" s="4" t="n"/>
+      <c r="I38" s="6" t="inlineStr"/>
+      <c r="J38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Mock-up (vliegtuigje)</t>
+          <t>Kabels en verbruik (in bezit)</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Arduino</t>
+          <t>Dupont-/siliconendraad</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Arduino Uno (heeft de gebruiker thuis)</t>
+          <t>Heeft de gebruiker</t>
         </is>
       </c>
       <c r="D39" s="7" t="n">
@@ -2013,30 +1898,26 @@
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
-      <c r="J39" s="6" t="inlineStr">
-        <is>
-          <t>Referentie antratek: Arduino Uno Rev3 (EUR 41,75)</t>
-        </is>
-      </c>
+      <c r="J39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>Mock-up (vliegtuigje)</t>
+          <t>Kabels en verbruik (in bezit)</t>
         </is>
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Servo's</t>
+          <t>USB A-kabel LoRa-ontvanger</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Bestaande voorraad (&gt; 3)</t>
+          <t>USB-A naar USB-C voor de XIAO (heeft de gebruiker)</t>
         </is>
       </c>
       <c r="D40" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E40" s="5" t="n"/>
       <c r="F40" s="5" t="n"/>
@@ -2056,17 +1937,17 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Mock-up (vliegtuigje)</t>
+          <t>Kabels en verbruik (in bezit)</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Servo-voeding</t>
+          <t>Gereedschap</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Aparte buck-converter</t>
+          <t>Schuifmaat, soldeerbout, tin, flux, multimeter, USB-serieel adapter</t>
         </is>
       </c>
       <c r="D41" s="7" t="n">
@@ -2087,319 +1968,365 @@
       <c r="I41" s="6" t="inlineStr"/>
       <c r="J41" s="6" t="inlineStr"/>
     </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>Mock-up (vliegtuigje)</t>
         </is>
       </c>
-      <c r="B42" s="6" t="inlineStr">
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
+      <c r="E42" s="4" t="n"/>
+      <c r="F42" s="4" t="n"/>
+      <c r="G42" s="4" t="n"/>
+      <c r="H42" s="4" t="n"/>
+      <c r="I42" s="4" t="n"/>
+      <c r="J42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Mock-up (vliegtuigje)</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Arduino</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Arduino Uno (heeft de gebruiker thuis)</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="14" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr"/>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>Referentie antratek: Arduino Uno Rev3 (EUR 41,75)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Mock-up (vliegtuigje)</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Servo's</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Bestaande voorraad (&gt; 3)</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="5" t="n"/>
+      <c r="G44" s="14" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I44" s="6" t="inlineStr"/>
+      <c r="J44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Mock-up (vliegtuigje)</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Servo-voeding</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Aparte buck-converter</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="n"/>
+      <c r="G45" s="14" t="inlineStr">
+        <is>
+          <t>al in bezit</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr"/>
+      <c r="J45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Mock-up (vliegtuigje)</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>Romp en roeren</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Eigen 3D-print</t>
         </is>
       </c>
-      <c r="D42" s="7" t="n">
+      <c r="D46" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E42" s="5" t="n"/>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="14" t="inlineStr">
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="5" t="n"/>
+      <c r="G46" s="14" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
       </c>
-      <c r="H42" s="5" t="inlineStr">
+      <c r="H46" s="5" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I42" s="6" t="inlineStr"/>
-      <c r="J42" s="6" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
+      <c r="I46" s="6" t="inlineStr"/>
+      <c r="J46" s="6" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="18" t="inlineStr">
         <is>
           <t>Totaal te bestellen bij Kiwi Electronics</t>
         </is>
       </c>
-      <c r="B44" s="20" t="n"/>
-      <c r="C44" s="20" t="n"/>
-      <c r="D44" s="20" t="n"/>
-      <c r="E44" s="20" t="n"/>
-      <c r="F44" s="21">
-        <f>SUMIF(G3:G42,"kiwi",F3:F42)</f>
+      <c r="B48" s="19" t="n"/>
+      <c r="C48" s="19" t="n"/>
+      <c r="D48" s="19" t="n"/>
+      <c r="E48" s="19" t="n"/>
+      <c r="F48" s="20">
+        <f>SUMIF(G3:G46,"kiwi",F3:F46)</f>
         <v/>
       </c>
-      <c r="G44" s="20" t="n"/>
-      <c r="H44" s="20" t="n"/>
-      <c r="I44" s="20" t="n"/>
-      <c r="J44" s="20" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="G48" s="19" t="n"/>
+      <c r="H48" s="19" t="n"/>
+      <c r="I48" s="19" t="n"/>
+      <c r="J48" s="19" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="inlineStr">
         <is>
           <t>Totaal te bestellen bij antratek</t>
         </is>
       </c>
-      <c r="B45" s="20" t="n"/>
-      <c r="C45" s="20" t="n"/>
-      <c r="D45" s="20" t="n"/>
-      <c r="E45" s="20" t="n"/>
-      <c r="F45" s="21">
-        <f>SUMIF(G3:G42,"antratek",F3:F42)</f>
+      <c r="B49" s="19" t="n"/>
+      <c r="C49" s="19" t="n"/>
+      <c r="D49" s="19" t="n"/>
+      <c r="E49" s="19" t="n"/>
+      <c r="F49" s="20">
+        <f>SUMIF(G3:G46,"antratek",F3:F46)</f>
         <v/>
       </c>
-      <c r="G45" s="20" t="n"/>
-      <c r="H45" s="20" t="n"/>
-      <c r="I45" s="20" t="n"/>
-      <c r="J45" s="20" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="19" t="inlineStr">
+      <c r="G49" s="19" t="n"/>
+      <c r="H49" s="19" t="n"/>
+      <c r="I49" s="19" t="n"/>
+      <c r="J49" s="19" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
         <is>
           <t>Totaal te bestellen bij AliExpress (China)</t>
         </is>
       </c>
-      <c r="B46" s="20" t="n"/>
-      <c r="C46" s="20" t="n"/>
-      <c r="D46" s="20" t="n"/>
-      <c r="E46" s="20" t="n"/>
-      <c r="F46" s="21">
-        <f>SUMIF(G3:G42,"aliexpress",F3:F42)</f>
+      <c r="B50" s="19" t="n"/>
+      <c r="C50" s="19" t="n"/>
+      <c r="D50" s="19" t="n"/>
+      <c r="E50" s="19" t="n"/>
+      <c r="F50" s="20">
+        <f>SUMIF(G3:G46,"aliexpress",F3:F46)</f>
         <v/>
       </c>
-      <c r="G46" s="20" t="n"/>
-      <c r="H46" s="20" t="n"/>
-      <c r="I46" s="20" t="n"/>
-      <c r="J46" s="20" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="19" t="inlineStr">
+      <c r="G50" s="19" t="n"/>
+      <c r="H50" s="19" t="n"/>
+      <c r="I50" s="19" t="n"/>
+      <c r="J50" s="19" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="18" t="inlineStr">
         <is>
           <t>Totaal te bestellen bij TME (EU)</t>
         </is>
       </c>
-      <c r="B47" s="20" t="n"/>
-      <c r="C47" s="20" t="n"/>
-      <c r="D47" s="20" t="n"/>
-      <c r="E47" s="20" t="n"/>
-      <c r="F47" s="21">
-        <f>SUMIF(G3:G42,"tme",F3:F42)</f>
+      <c r="B51" s="19" t="n"/>
+      <c r="C51" s="19" t="n"/>
+      <c r="D51" s="19" t="n"/>
+      <c r="E51" s="19" t="n"/>
+      <c r="F51" s="20">
+        <f>SUMIF(G3:G46,"tme",F3:F46)</f>
         <v/>
       </c>
-      <c r="G47" s="20" t="n"/>
-      <c r="H47" s="20" t="n"/>
-      <c r="I47" s="20" t="n"/>
-      <c r="J47" s="20" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="19" t="inlineStr">
+      <c r="G51" s="19" t="n"/>
+      <c r="H51" s="19" t="n"/>
+      <c r="I51" s="19" t="n"/>
+      <c r="J51" s="19" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="18" t="inlineStr">
         <is>
           <t>Totaal te bestellen bij Mouser/DigiKey (EU)</t>
         </is>
       </c>
-      <c r="B48" s="20" t="n"/>
-      <c r="C48" s="20" t="n"/>
-      <c r="D48" s="20" t="n"/>
-      <c r="E48" s="20" t="n"/>
-      <c r="F48" s="21">
-        <f>SUMIF(G3:G42,"mouser",F3:F42)</f>
+      <c r="B52" s="19" t="n"/>
+      <c r="C52" s="19" t="n"/>
+      <c r="D52" s="19" t="n"/>
+      <c r="E52" s="19" t="n"/>
+      <c r="F52" s="20">
+        <f>SUMIF(G3:G46,"mouser",F3:F46)</f>
         <v/>
       </c>
-      <c r="G48" s="20" t="n"/>
-      <c r="H48" s="20" t="n"/>
-      <c r="I48" s="20" t="n"/>
-      <c r="J48" s="20" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="19" t="inlineStr">
-        <is>
-          <t>Totaal te bestellen bij HESTORE (EU)</t>
-        </is>
-      </c>
-      <c r="B49" s="20" t="n"/>
-      <c r="C49" s="20" t="n"/>
-      <c r="D49" s="20" t="n"/>
-      <c r="E49" s="20" t="n"/>
-      <c r="F49" s="21">
-        <f>SUMIF(G3:G42,"hestore",F3:F42)</f>
+      <c r="G52" s="19" t="n"/>
+      <c r="H52" s="19" t="n"/>
+      <c r="I52" s="19" t="n"/>
+      <c r="J52" s="19" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="18" t="inlineStr">
+        <is>
+          <t>Waveshare: losse GNSS-antenne (voorwaardelijk)</t>
+        </is>
+      </c>
+      <c r="B53" s="19" t="n"/>
+      <c r="C53" s="19" t="n"/>
+      <c r="D53" s="19" t="n"/>
+      <c r="E53" s="19" t="n"/>
+      <c r="F53" s="20">
+        <f>SUMIF(G3:G46,"waveshare",F3:F46)</f>
         <v/>
       </c>
-      <c r="G49" s="20" t="n"/>
-      <c r="H49" s="20" t="n"/>
-      <c r="I49" s="20" t="n"/>
-      <c r="J49" s="20" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="19" t="inlineStr">
-        <is>
-          <t>Totaal te bestellen bij TinyTronics (NL)</t>
-        </is>
-      </c>
-      <c r="B50" s="20" t="n"/>
-      <c r="C50" s="20" t="n"/>
-      <c r="D50" s="20" t="n"/>
-      <c r="E50" s="20" t="n"/>
-      <c r="F50" s="21">
-        <f>SUMIF(G3:G42,"tinytronics",F3:F42)</f>
+      <c r="G53" s="19" t="n"/>
+      <c r="H53" s="19" t="n"/>
+      <c r="I53" s="19" t="n"/>
+      <c r="J53" s="19" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>Eckstein-terugvaloptie (niet gekozen; geen actieve regel)</t>
+        </is>
+      </c>
+      <c r="B54" s="19" t="n"/>
+      <c r="C54" s="19" t="n"/>
+      <c r="D54" s="19" t="n"/>
+      <c r="E54" s="19" t="n"/>
+      <c r="F54" s="20">
+        <f>SUMIF(G3:G46,"eckstein",F3:F46)</f>
         <v/>
       </c>
-      <c r="G50" s="20" t="n"/>
-      <c r="H50" s="20" t="n"/>
-      <c r="I50" s="20" t="n"/>
-      <c r="J50" s="20" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="19" t="inlineStr">
-        <is>
-          <t>Waveshare: losse GNSS-antenne (voorwaardelijk)</t>
-        </is>
-      </c>
-      <c r="B51" s="20" t="n"/>
-      <c r="C51" s="20" t="n"/>
-      <c r="D51" s="20" t="n"/>
-      <c r="E51" s="20" t="n"/>
-      <c r="F51" s="21">
-        <f>SUMIF(G3:G42,"waveshare",F3:F42)</f>
+      <c r="G54" s="19" t="n"/>
+      <c r="H54" s="19" t="n"/>
+      <c r="I54" s="19" t="n"/>
+      <c r="J54" s="19" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="18" t="inlineStr">
+        <is>
+          <t>TOTAAL actieve onderdelen (incl. voorwaardelijke GNSS-antenne)</t>
+        </is>
+      </c>
+      <c r="B55" s="19" t="n"/>
+      <c r="C55" s="19" t="n"/>
+      <c r="D55" s="19" t="n"/>
+      <c r="E55" s="19" t="n"/>
+      <c r="F55" s="20">
+        <f>SUM(F3:F46)</f>
         <v/>
       </c>
-      <c r="G51" s="20" t="n"/>
-      <c r="H51" s="20" t="n"/>
-      <c r="I51" s="20" t="n"/>
-      <c r="J51" s="20" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="19" t="inlineStr">
-        <is>
-          <t>Eckstein-terugvaloptie (niet gekozen; geen actieve regel)</t>
-        </is>
-      </c>
-      <c r="B52" s="20" t="n"/>
-      <c r="C52" s="20" t="n"/>
-      <c r="D52" s="20" t="n"/>
-      <c r="E52" s="20" t="n"/>
-      <c r="F52" s="21">
-        <f>SUMIF(G3:G42,"eckstein",F3:F42)</f>
+      <c r="G55" s="19" t="n"/>
+      <c r="H55" s="19" t="n"/>
+      <c r="I55" s="19" t="n"/>
+      <c r="J55" s="19" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="18" t="inlineStr">
+        <is>
+          <t>TOTAAL actieve onderdelen excl. losse GNSS-antenne</t>
+        </is>
+      </c>
+      <c r="B56" s="19" t="n"/>
+      <c r="C56" s="19" t="n"/>
+      <c r="D56" s="19" t="n"/>
+      <c r="E56" s="19" t="n"/>
+      <c r="F56" s="20">
+        <f>F55-F53</f>
         <v/>
       </c>
-      <c r="G52" s="20" t="n"/>
-      <c r="H52" s="20" t="n"/>
-      <c r="I52" s="20" t="n"/>
-      <c r="J52" s="20" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="19" t="inlineStr">
-        <is>
-          <t>TOTAAL alle onderdelen excl. AISLER-print (incl. losse antenne)</t>
-        </is>
-      </c>
-      <c r="B53" s="20" t="n"/>
-      <c r="C53" s="20" t="n"/>
-      <c r="D53" s="20" t="n"/>
-      <c r="E53" s="20" t="n"/>
-      <c r="F53" s="21">
-        <f>SUM(F3:F42)-SUMIF(G3:G42,"aisler",F3:F42)</f>
-        <v/>
-      </c>
-      <c r="G53" s="20" t="n"/>
-      <c r="H53" s="20" t="n"/>
-      <c r="I53" s="20" t="n"/>
-      <c r="J53" s="20" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="19" t="inlineStr">
-        <is>
-          <t>TOTAAL onderdelen excl. losse GNSS-antenne (excl. AISLER)</t>
-        </is>
-      </c>
-      <c r="B54" s="20" t="n"/>
-      <c r="C54" s="20" t="n"/>
-      <c r="D54" s="20" t="n"/>
-      <c r="E54" s="20" t="n"/>
-      <c r="F54" s="21">
-        <f>F53-F51</f>
-        <v/>
-      </c>
-      <c r="G54" s="20" t="n"/>
-      <c r="H54" s="20" t="n"/>
-      <c r="I54" s="20" t="n"/>
-      <c r="J54" s="20" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="19" t="inlineStr">
-        <is>
-          <t>Totaal draagprint bij AISLER (3 stuks)</t>
-        </is>
-      </c>
-      <c r="B55" s="20" t="n"/>
-      <c r="C55" s="20" t="n"/>
-      <c r="D55" s="20" t="n"/>
-      <c r="E55" s="20" t="n"/>
-      <c r="F55" s="21">
-        <f>SUMIF(G3:G42,"aisler",F3:F42)</f>
-        <v/>
-      </c>
-      <c r="G55" s="20" t="n"/>
-      <c r="H55" s="20" t="n"/>
-      <c r="I55" s="20" t="n"/>
-      <c r="J55" s="20" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="19" t="inlineStr">
-        <is>
-          <t>TOTAAL alles (incl. losse antenne + AISLER-print)</t>
-        </is>
-      </c>
-      <c r="B56" s="20" t="n"/>
-      <c r="C56" s="20" t="n"/>
-      <c r="D56" s="20" t="n"/>
-      <c r="E56" s="20" t="n"/>
-      <c r="F56" s="21">
-        <f>F53+F55</f>
-        <v/>
-      </c>
-      <c r="G56" s="20" t="n"/>
-      <c r="H56" s="20" t="n"/>
-      <c r="I56" s="20" t="n"/>
-      <c r="J56" s="20" t="n"/>
+      <c r="G56" s="19" t="n"/>
+      <c r="H56" s="19" t="n"/>
+      <c r="I56" s="19" t="n"/>
+      <c r="J56" s="19" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="22" t="inlineStr">
-        <is>
-          <t>Let op: prijzen zijn onder voorbehoud en incl. btw. Bij de AliExpress-GPS moet je de LC29HDA (rover)-variant kiezen, geen LC29HBS (basisstation) en geen losse SMD-module. De losse Waveshare-antenne (SKU 25346) is voorwaardelijk: eerst checken of de boardkit een passende L1/L5-antenne meelevert. Terugvaloptie GPS in de EU: Waveshare LC29H(DA) HAT (Eckstein ca. EUR 71,39 / Kamami ca. EUR 63). De LED + 330 Ohm-weerstand (10-packs) heeft de gebruiker thuis en is dus niet meer te bestellen. Zie GEBRUIKER/data/bestelbaarheid.md en GEBRUIKER/data/bestelschema-pcb.md.</t>
+      <c r="A58" s="21" t="inlineStr">
+        <is>
+          <t>Let op: prijzen zijn onder voorbehoud en incl. btw. Bij de AliExpress-GPS moet je de LC29HDA (rover)-variant kiezen, geen LC29HBS (basisstation) en geen losse SMD-module. De losse Waveshare-antenne (SKU 25346) is voorwaardelijk: eerst checken of de boardkit een passende L1/L5-antenne meelevert. Terugvaloptie GPS in de EU: Waveshare LC29H(DA) HAT (Eckstein ca. EUR 71,39 / Kamami ca. EUR 63). De LED + 330 Ohm-weerstand (10-packs) heeft de gebruiker thuis en is dus niet meer te bestellen. Carrier-PCB en sockets zijn vervallen; montage- en connectorbehoefte is nog te bepalen. Zie GEBRUIKER/data/bedrading-en-behuizing.md.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:J42"/>
+  <autoFilter ref="A2:J46"/>
   <mergeCells count="22">
     <mergeCell ref="A5:J5"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A22:J22"/>
     <mergeCell ref="A49:E49"/>
     <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A45:E45"/>
-    <mergeCell ref="A38:J38"/>
+    <mergeCell ref="A29:J29"/>
     <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A31:J31"/>
     <mergeCell ref="A54:E54"/>
     <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A46:E46"/>
     <mergeCell ref="A24:J24"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A50:E50"/>
     <mergeCell ref="A55:E55"/>
-    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A16:J16"/>
     <mergeCell ref="A53:E53"/>
+    <mergeCell ref="A37:J37"/>
     <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A18:J18"/>
     <mergeCell ref="A3:J3"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A33:J33"/>
+    <mergeCell ref="A26:J26"/>
+    <mergeCell ref="A42:J42"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I4" r:id="rId1"/>
@@ -2408,16 +2335,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2429,7 +2351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2437,19 +2359,19 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>Betekenis</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>kiwi</t>
         </is>
@@ -2461,7 +2383,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="24" t="inlineStr">
         <is>
           <t>antratek</t>
         </is>
@@ -2473,7 +2395,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>aliexpress</t>
         </is>
@@ -2485,7 +2407,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="26" t="inlineStr">
         <is>
           <t>waveshare</t>
         </is>
@@ -2497,7 +2419,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>eckstein</t>
         </is>
@@ -2509,19 +2431,19 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>tme</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TME (Polen, EU): LDO, TVS, schroefklem, precisie-sockets</t>
+          <t>TME (Polen, EU): eerder gekozen LDO/TVS; montage van de componenten nog open</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>mouser</t>
         </is>
@@ -2533,108 +2455,120 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>niet nodig</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bewust niet voorzien (bv. P-MOSFET-ompoolbeveiliging, beslissing 2026-10-06)</t>
+          <t>Niet bestellen of bewust niet voorzien; o.a. carrier-PCB en sockets vervallen (2026-10-09)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>te bepalen</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Montage- of connectorbehoefte nog open; niet opgenomen in actieve totalen</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>hestore</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>HESTORE (Hongarije, EU): schroefklem DEGSON</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HESTORE (Hongarije, EU): historische schroefklemoptie; niet meer actief besteld</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>tinytronics</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>TinyTronics (Nederland, EU): M3-montagesets</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="32" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>TinyTronics (Nederland, EU): historische M3-set voor oude printmontage</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>aisler</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Gefabriceerd bij AISLER (EU); print zelf, geen componenten</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Historische fabrikant van de vervallen carrier-PCB; niet bestellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t>schatting</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Prijs is een schatting; apart te bestellen bij een componentenwinkel</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="33" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>al in bezit</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Heeft de gebruiker al; niet aankopen</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="34" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>geen link</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Niet gevonden bij Kiwi of antratek; nog geen prijs</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
         <is>
           <t>onderzoek</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Zoekrichting bekend, maar productlisting/prijs nog niet gevalideerd</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>niet nodig</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Bewust niet voorzien</t>
         </is>
@@ -2651,7 +2585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2661,23 +2595,23 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
-        <is>
-          <t>Bestelschema draagprint bij AISLER - schatting (2026-10-06)</t>
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>Bedrading en montage - open keuzes (2026-10-09)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="36" t="inlineStr">
-        <is>
-          <t>AISLER-productie - 2-laags 1,6 mm HASL Budget</t>
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>Huidige aanpak: handbedrading en behuizing</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Formule: EUR 12,00 job fee + EUR 0,067/cm2 x oppervlak x aantal (sets van 3, gratis verzending, productie vanaf 2 werkdagen)</t>
+          <t>Geen eigen carrier-PCB en geen socket-headers. De gebruiker bedradt en soldeert zelf; de onderdelen worden aan een 3D-geprinte behuizing gemonteerd.</t>
         </is>
       </c>
       <c r="B3" s="6" t="n"/>
@@ -2685,116 +2619,134 @@
       <c r="D3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="37" t="inlineStr">
-        <is>
-          <t>Oppervlak</t>
-        </is>
-      </c>
-      <c r="B4" s="37" t="inlineStr">
-        <is>
-          <t>3 stuks incl. btw</t>
-        </is>
-      </c>
-      <c r="C4" s="37" t="inlineStr">
-        <is>
-          <t>6 stuks incl. btw</t>
-        </is>
-      </c>
-      <c r="D4" s="37" t="n"/>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Breakoutmodules</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Blijven behouden</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Zelf bedraden; exacte verbindingen nog uit te werken</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>60 cm2 (bv. 100x60)</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>29.11</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>43.71</v>
+          <t>Montagehardware</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Nog te bepalen</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Niet toevoegen of online opzoeken voordat montagewijze bevestigd is</t>
+        </is>
       </c>
       <c r="D5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>75 cm2 (100x75, aanname)</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>32.76</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>50.99</v>
+          <t>UART-/uitbreidingsconnector</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Nog te bepalen</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Eerder gekozen schroefklem kan vervallen bij rechtstreeks bedraden</t>
+        </is>
       </c>
       <c r="D6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>90 cm2 (120x75)</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>36.41</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>58.3</v>
+          <t>Voedingsinvoer</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Nog te bepalen</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Bestaande barrel-adapter aanwezig; paneel-/behuizingsmontage open</t>
+        </is>
       </c>
       <c r="D7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>100 cm2 (100x100)</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>38.84</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>63.16</v>
+          <t>PTC, TVS, LDO en ontkoppeling</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Functies voorlopig behouden</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Handbedrading en mechanische ondersteuning nog uit te werken</t>
+        </is>
       </c>
       <c r="D8" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="inlineStr">
-        <is>
-          <t>Onderdelen op de print (gevonden bij EU-winkels, 2026-10-06)</t>
+      <c r="A10" s="35" t="inlineStr">
+        <is>
+          <t>Vervallen bestellingen</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="37" t="inlineStr">
-        <is>
-          <t>Onderdeel</t>
-        </is>
-      </c>
-      <c r="B11" s="37" t="inlineStr">
-        <is>
-          <t>Prijs (EUR)</t>
-        </is>
-      </c>
-      <c r="C11" s="37" t="inlineStr">
-        <is>
-          <t>Leverancier</t>
-        </is>
-      </c>
-      <c r="D11" s="37" t="n"/>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Carrier-PCB bij AISLER</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Niet nodig</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Geen print produceren of bestellen</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Sockets: dual-wipe + Preci-Dip turned-pin</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n">
-        <v>5</v>
+          <t>Socket-headers</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Niet nodig</t>
+        </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>TME / RS Components</t>
+          <t>Breakoutmodules worden met draden aangesloten en gesoldeerd</t>
         </is>
       </c>
       <c r="D12" s="6" t="n"/>
@@ -2802,15 +2754,17 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>PTC Littelfuse 1812L200/16 + TVS SMBJ10A-TR (zonder P-MOSFET)</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="n">
-        <v>1</v>
+          <t>PCB-barreljack</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>Niet nodig</t>
+        </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Mouser.be / DigiKey (EU)</t>
+          <t>Specifiek gekozen voor montage op de vervallen PCB</t>
         </is>
       </c>
       <c r="D13" s="6" t="n"/>
@@ -2818,304 +2772,84 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>LDO AP2112K-3.3TRG1</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="n">
-        <v>0.27</v>
+          <t>Oude M3-set</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Niet actief</t>
+        </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>TME (EU)</t>
+          <t>Was bedoeld voor printmontage; behuizingsbevestiging nog te bepalen</t>
         </is>
       </c>
       <c r="D14" s="6" t="n"/>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Schroefklem 4-pins 3,5 mm DEGSON DG250-3.5-04P</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>HESTORE / TME (EU)</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n"/>
-    </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>M3-schroeven, moeren, afstandsbusjes, spacers</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n">
-        <v>8</v>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>TinyTronics (NL, EU)</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="n"/>
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>Vervolgstappen (geen nieuwe aankopen vastgelegd)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="37" t="inlineStr">
-        <is>
-          <t>Subtotaal apart te bestellen</t>
-        </is>
-      </c>
-      <c r="B17" s="38" t="n">
-        <v>14.88</v>
-      </c>
-      <c r="C17" s="37" t="inlineStr">
-        <is>
-          <t>EU-winkels</t>
-        </is>
-      </c>
-      <c r="D17" s="37" t="n"/>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>1. Bevestig hoe de breakoutmodules en losse componenten aan de behuizing worden gemonteerd</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>TXB0108 level shifter</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="n">
-        <v>8.699999999999999</v>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
+          <t>2. Werk bedradingsroute, isolatie/ondersteuning en trekontlasting uit</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
       <c r="D18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>Power-LED + serieweerstand (10-packs thuis in bezit)</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>Heeft de gebruiker</t>
-        </is>
-      </c>
+          <t>3. Bevestig of de UART-klem en voedingsaansluiting nodig blijven</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
       <c r="D19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Ontkoppelcondensatoren (per bord gebruikt)</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
+          <t>4. Controleer of aanwezige draad en printmateriaal volstaan; koop niets nieuws zonder bevestiging</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>Bulk-elco 100 uF</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
+          <t>5. Herbereken de bestellijst nadat de montagekeuzes vastliggen</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
       <c r="D21" s="6" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="37" t="inlineStr">
-        <is>
-          <t>Subtotaal al in hoofd-bestellijst</t>
-        </is>
-      </c>
-      <c r="B22" s="38" t="n">
-        <v>9.789999999999999</v>
-      </c>
-      <c r="C22" s="37" t="inlineStr">
-        <is>
-          <t>Kiwi Electronics</t>
-        </is>
-      </c>
-      <c r="D22" s="37" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="37" t="inlineStr">
-        <is>
-          <t>Totaal onderdelen op de print (met TXB0108)</t>
-        </is>
-      </c>
-      <c r="B23" s="38" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="C23" s="37" t="inlineStr">
-        <is>
-          <t>met TXB0104-IC direct: ca. 17,77</t>
-        </is>
-      </c>
-      <c r="D23" s="37" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="36" t="inlineStr">
-        <is>
-          <t>Totalen (3 borden, incl. btw)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>AISLER print, 3 stuks, 75 cm2 Budget</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n">
-        <v>32.76</v>
-      </c>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Onderdelen op de print</t>
-        </is>
-      </c>
-      <c r="B27" s="8" t="n">
-        <v>24.67</v>
-      </c>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="37" t="inlineStr">
-        <is>
-          <t>Totaal</t>
-        </is>
-      </c>
-      <c r="B28" s="38" t="n">
-        <v>57.43</v>
-      </c>
-      <c r="C28" s="37" t="n"/>
-      <c r="D28" s="37" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>Waarvan al in de hoofd-bestellijst</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="n">
-        <v>9.789999999999999</v>
-      </c>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="37" t="inlineStr">
-        <is>
-          <t>Werkelijk nieuw te bestellen</t>
-        </is>
-      </c>
-      <c r="B30" s="38" t="n">
-        <v>47.64</v>
-      </c>
-      <c r="C30" s="37" t="n"/>
-      <c r="D30" s="37" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="36" t="inlineStr">
-        <is>
-          <t>Bestelvolgorde</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>1. PCB ontwerpen in KiCad; layout afronden, DRC, Gerbers/ODB++ exporteren</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>2. Bordafmeting definitief nameten en AISLER-calculator controleren</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>3. Print bestellen bij AISLER (3 of 6 stuks, Budget-service)</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>4. Tegelijk de printonderdelen bij EU-winkels bestellen (TME, Mouser, HESTORE, TinyTronics)</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="6" t="n"/>
-      <c r="D36" s="6" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>5. Kiwi/antratek-bestelling: level shifter, condensatoren, bulk-elco (LED + 330 Ohm heeft de gebruiker thuis)</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>6. Rendering vergelijken met het echte bord, daarna solderen</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A32:D32"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3137,29 +2871,29 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
-        <is>
-          <t>Bestelbaarheid - gecontroleerd op 2026-10-06</t>
+      <c r="A1" s="34" t="inlineStr">
+        <is>
+          <t>Bestelbaarheid - historische controle op 2026-10-06 (geen actuele besteladviezen)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Winkel</t>
         </is>
       </c>
-      <c r="B2" s="23" t="inlineStr">
+      <c r="B2" s="22" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
+      <c r="C2" s="22" t="inlineStr">
         <is>
           <t>Voorraad</t>
         </is>
       </c>
-      <c r="D2" s="23" t="inlineStr">
+      <c r="D2" s="22" t="inlineStr">
         <is>
           <t>Opmerking</t>
         </is>
@@ -3475,7 +3209,7 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>niet in kleine aantallen</t>
+          <t>historische regel; sockets vervallen op 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3275,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>EUR 8,00 incl.</t>
+          <t>historische prijs; bedoeld voor de vervallen PCB-montage</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3297,7 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>EUR 6,95 incl.</t>
+          <t>historische prijs; montage voor behuizing nog te bepalen</t>
         </is>
       </c>
     </row>

</xml_diff>